<commit_message>
finance case update - model automation - correct input
</commit_message>
<xml_diff>
--- a/cases/finance/model.xlsx
+++ b/cases/finance/model.xlsx
@@ -14,69 +14,90 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="in_revenue_2026_02">Inputs!$B$2</definedName>
-    <definedName name="in_revenue_2026_03">Inputs!$C$2</definedName>
-    <definedName name="in_revenue_2026_04">Inputs!$D$2</definedName>
-    <definedName name="in_cogs_2026_02">Inputs!$B$3</definedName>
-    <definedName name="in_cogs_2026_03">Inputs!$C$3</definedName>
-    <definedName name="in_cogs_2026_04">Inputs!$D$3</definedName>
-    <definedName name="in_sganda_2026_02">Inputs!$B$4</definedName>
-    <definedName name="in_sganda_2026_03">Inputs!$C$4</definedName>
-    <definedName name="in_sganda_2026_04">Inputs!$D$4</definedName>
-    <definedName name="in_randd_2026_02">Inputs!$B$5</definedName>
-    <definedName name="in_randd_2026_03">Inputs!$C$5</definedName>
-    <definedName name="in_randd_2026_04">Inputs!$D$5</definedName>
-    <definedName name="in_depreciation_2026_02">Inputs!$B$6</definedName>
-    <definedName name="in_depreciation_2026_03">Inputs!$C$6</definedName>
-    <definedName name="in_depreciation_2026_04">Inputs!$D$6</definedName>
-    <definedName name="in_interest_expense_2026_02">Inputs!$B$7</definedName>
-    <definedName name="in_interest_expense_2026_03">Inputs!$C$7</definedName>
-    <definedName name="in_interest_expense_2026_04">Inputs!$D$7</definedName>
-    <definedName name="in_interest_income_2026_02">Inputs!$B$8</definedName>
-    <definedName name="in_interest_income_2026_03">Inputs!$C$8</definedName>
-    <definedName name="in_interest_income_2026_04">Inputs!$D$8</definedName>
-    <definedName name="in_tax_expense_2026_02">Inputs!$B$9</definedName>
-    <definedName name="in_tax_expense_2026_03">Inputs!$C$9</definedName>
-    <definedName name="in_tax_expense_2026_04">Inputs!$D$9</definedName>
-    <definedName name="in_cash_2026_02">Inputs!$B$10</definedName>
-    <definedName name="in_cash_2026_03">Inputs!$C$10</definedName>
-    <definedName name="in_cash_2026_04">Inputs!$D$10</definedName>
-    <definedName name="in_ar_2026_02">Inputs!$B$11</definedName>
-    <definedName name="in_ar_2026_03">Inputs!$C$11</definedName>
-    <definedName name="in_ar_2026_04">Inputs!$D$11</definedName>
-    <definedName name="in_inventory_2026_02">Inputs!$B$12</definedName>
-    <definedName name="in_inventory_2026_03">Inputs!$C$12</definedName>
-    <definedName name="in_inventory_2026_04">Inputs!$D$12</definedName>
-    <definedName name="in_prepaid_expenses_2026_02">Inputs!$B$13</definedName>
-    <definedName name="in_prepaid_expenses_2026_03">Inputs!$C$13</definedName>
-    <definedName name="in_prepaid_expenses_2026_04">Inputs!$D$13</definedName>
-    <definedName name="in_ppe_2026_02">Inputs!$B$14</definedName>
-    <definedName name="in_ppe_2026_03">Inputs!$C$14</definedName>
-    <definedName name="in_ppe_2026_04">Inputs!$D$14</definedName>
-    <definedName name="in_intangibles_2026_02">Inputs!$B$15</definedName>
-    <definedName name="in_intangibles_2026_03">Inputs!$C$15</definedName>
-    <definedName name="in_intangibles_2026_04">Inputs!$D$15</definedName>
-    <definedName name="in_ap_2026_02">Inputs!$B$16</definedName>
-    <definedName name="in_ap_2026_03">Inputs!$C$16</definedName>
-    <definedName name="in_ap_2026_04">Inputs!$D$16</definedName>
-    <definedName name="in_accrued_expenses_2026_02">Inputs!$B$17</definedName>
-    <definedName name="in_accrued_expenses_2026_03">Inputs!$C$17</definedName>
-    <definedName name="in_accrued_expenses_2026_04">Inputs!$D$17</definedName>
-    <definedName name="in_lease_liability_st_2026_02">Inputs!$B$18</definedName>
-    <definedName name="in_lease_liability_st_2026_03">Inputs!$C$18</definedName>
-    <definedName name="in_lease_liability_st_2026_04">Inputs!$D$18</definedName>
-    <definedName name="in_lease_liability_lt_2026_02">Inputs!$B$19</definedName>
-    <definedName name="in_lease_liability_lt_2026_03">Inputs!$C$19</definedName>
-    <definedName name="in_lease_liability_lt_2026_04">Inputs!$D$19</definedName>
-    <definedName name="in_debt_2026_02">Inputs!$B$20</definedName>
-    <definedName name="in_debt_2026_03">Inputs!$C$20</definedName>
-    <definedName name="in_debt_2026_04">Inputs!$D$20</definedName>
-    <definedName name="in_common_stock_2026_02">Inputs!$B$21</definedName>
-    <definedName name="in_common_stock_2026_03">Inputs!$C$21</definedName>
-    <definedName name="in_common_stock_2026_04">Inputs!$D$21</definedName>
-    <definedName name="in_retained_earnings_prior_2026_02">Inputs!$B$22</definedName>
-    <definedName name="in_retained_earnings_prior_2026_03">Inputs!$C$22</definedName>
-    <definedName name="in_retained_earnings_prior_2026_04">Inputs!$D$22</definedName>
+    <definedName name="in_revenue_2026_01">Inputs!$B$2</definedName>
+    <definedName name="in_revenue_2026_02">Inputs!$C$2</definedName>
+    <definedName name="in_revenue_2026_03">Inputs!$D$2</definedName>
+    <definedName name="in_revenue_2026_04">Inputs!$E$2</definedName>
+    <definedName name="in_cogs_2026_01">Inputs!$B$3</definedName>
+    <definedName name="in_cogs_2026_02">Inputs!$C$3</definedName>
+    <definedName name="in_cogs_2026_03">Inputs!$D$3</definedName>
+    <definedName name="in_cogs_2026_04">Inputs!$E$3</definedName>
+    <definedName name="in_sganda_2026_01">Inputs!$B$4</definedName>
+    <definedName name="in_sganda_2026_02">Inputs!$C$4</definedName>
+    <definedName name="in_sganda_2026_03">Inputs!$D$4</definedName>
+    <definedName name="in_sganda_2026_04">Inputs!$E$4</definedName>
+    <definedName name="in_randd_2026_01">Inputs!$B$5</definedName>
+    <definedName name="in_randd_2026_02">Inputs!$C$5</definedName>
+    <definedName name="in_randd_2026_03">Inputs!$D$5</definedName>
+    <definedName name="in_randd_2026_04">Inputs!$E$5</definedName>
+    <definedName name="in_depreciation_2026_01">Inputs!$B$6</definedName>
+    <definedName name="in_depreciation_2026_02">Inputs!$C$6</definedName>
+    <definedName name="in_depreciation_2026_03">Inputs!$D$6</definedName>
+    <definedName name="in_depreciation_2026_04">Inputs!$E$6</definedName>
+    <definedName name="in_interest_expense_2026_01">Inputs!$B$7</definedName>
+    <definedName name="in_interest_expense_2026_02">Inputs!$C$7</definedName>
+    <definedName name="in_interest_expense_2026_03">Inputs!$D$7</definedName>
+    <definedName name="in_interest_expense_2026_04">Inputs!$E$7</definedName>
+    <definedName name="in_interest_income_2026_01">Inputs!$B$8</definedName>
+    <definedName name="in_interest_income_2026_02">Inputs!$C$8</definedName>
+    <definedName name="in_interest_income_2026_03">Inputs!$D$8</definedName>
+    <definedName name="in_interest_income_2026_04">Inputs!$E$8</definedName>
+    <definedName name="in_tax_expense_2026_01">Inputs!$B$9</definedName>
+    <definedName name="in_tax_expense_2026_02">Inputs!$C$9</definedName>
+    <definedName name="in_tax_expense_2026_03">Inputs!$D$9</definedName>
+    <definedName name="in_tax_expense_2026_04">Inputs!$E$9</definedName>
+    <definedName name="in_cash_2026_01">Inputs!$B$10</definedName>
+    <definedName name="in_cash_2026_02">Inputs!$C$10</definedName>
+    <definedName name="in_cash_2026_03">Inputs!$D$10</definedName>
+    <definedName name="in_cash_2026_04">Inputs!$E$10</definedName>
+    <definedName name="in_ar_2026_01">Inputs!$B$11</definedName>
+    <definedName name="in_ar_2026_02">Inputs!$C$11</definedName>
+    <definedName name="in_ar_2026_03">Inputs!$D$11</definedName>
+    <definedName name="in_ar_2026_04">Inputs!$E$11</definedName>
+    <definedName name="in_inventory_2026_01">Inputs!$B$12</definedName>
+    <definedName name="in_inventory_2026_02">Inputs!$C$12</definedName>
+    <definedName name="in_inventory_2026_03">Inputs!$D$12</definedName>
+    <definedName name="in_inventory_2026_04">Inputs!$E$12</definedName>
+    <definedName name="in_prepaid_expenses_2026_01">Inputs!$B$13</definedName>
+    <definedName name="in_prepaid_expenses_2026_02">Inputs!$C$13</definedName>
+    <definedName name="in_prepaid_expenses_2026_03">Inputs!$D$13</definedName>
+    <definedName name="in_prepaid_expenses_2026_04">Inputs!$E$13</definedName>
+    <definedName name="in_ppe_2026_01">Inputs!$B$14</definedName>
+    <definedName name="in_ppe_2026_02">Inputs!$C$14</definedName>
+    <definedName name="in_ppe_2026_03">Inputs!$D$14</definedName>
+    <definedName name="in_ppe_2026_04">Inputs!$E$14</definedName>
+    <definedName name="in_intangibles_2026_01">Inputs!$B$15</definedName>
+    <definedName name="in_intangibles_2026_02">Inputs!$C$15</definedName>
+    <definedName name="in_intangibles_2026_03">Inputs!$D$15</definedName>
+    <definedName name="in_intangibles_2026_04">Inputs!$E$15</definedName>
+    <definedName name="in_ap_2026_01">Inputs!$B$16</definedName>
+    <definedName name="in_ap_2026_02">Inputs!$C$16</definedName>
+    <definedName name="in_ap_2026_03">Inputs!$D$16</definedName>
+    <definedName name="in_ap_2026_04">Inputs!$E$16</definedName>
+    <definedName name="in_accrued_expenses_2026_01">Inputs!$B$17</definedName>
+    <definedName name="in_accrued_expenses_2026_02">Inputs!$C$17</definedName>
+    <definedName name="in_accrued_expenses_2026_03">Inputs!$D$17</definedName>
+    <definedName name="in_accrued_expenses_2026_04">Inputs!$E$17</definedName>
+    <definedName name="in_lease_liability_st_2026_01">Inputs!$B$18</definedName>
+    <definedName name="in_lease_liability_st_2026_02">Inputs!$C$18</definedName>
+    <definedName name="in_lease_liability_st_2026_03">Inputs!$D$18</definedName>
+    <definedName name="in_lease_liability_st_2026_04">Inputs!$E$18</definedName>
+    <definedName name="in_lease_liability_lt_2026_01">Inputs!$B$19</definedName>
+    <definedName name="in_lease_liability_lt_2026_02">Inputs!$C$19</definedName>
+    <definedName name="in_lease_liability_lt_2026_03">Inputs!$D$19</definedName>
+    <definedName name="in_lease_liability_lt_2026_04">Inputs!$E$19</definedName>
+    <definedName name="in_debt_2026_01">Inputs!$B$20</definedName>
+    <definedName name="in_debt_2026_02">Inputs!$C$20</definedName>
+    <definedName name="in_debt_2026_03">Inputs!$D$20</definedName>
+    <definedName name="in_debt_2026_04">Inputs!$E$20</definedName>
+    <definedName name="in_common_stock_2026_01">Inputs!$B$21</definedName>
+    <definedName name="in_common_stock_2026_02">Inputs!$C$21</definedName>
+    <definedName name="in_common_stock_2026_03">Inputs!$D$21</definedName>
+    <definedName name="in_common_stock_2026_04">Inputs!$E$21</definedName>
+    <definedName name="in_retained_earnings_prior_2026_01">Inputs!$B$22</definedName>
+    <definedName name="in_retained_earnings_prior_2026_02">Inputs!$C$22</definedName>
+    <definedName name="in_retained_earnings_prior_2026_03">Inputs!$D$22</definedName>
+    <definedName name="in_retained_earnings_prior_2026_04">Inputs!$E$22</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -107,7 +128,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +138,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -132,12 +158,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,13 +534,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -524,15 +552,20 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -551,8 +584,9 @@
         <v>2690522.54</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2735888.82</v>
-      </c>
+        <v>2734888.82</v>
+      </c>
+      <c r="E2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -569,6 +603,7 @@
       <c r="D3" s="3" t="n">
         <v>-1506936.06</v>
       </c>
+      <c r="E3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -583,8 +618,9 @@
         <v>-543642.53</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>-557644.4</v>
-      </c>
+        <v>-556144.4</v>
+      </c>
+      <c r="E4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -601,6 +637,7 @@
       <c r="D5" s="3" t="n">
         <v>-196346.72</v>
       </c>
+      <c r="E5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -617,6 +654,7 @@
       <c r="D6" s="3" t="n">
         <v>-61592.78</v>
       </c>
+      <c r="E6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -633,6 +671,7 @@
       <c r="D7" s="3" t="n">
         <v>-19352.6</v>
       </c>
+      <c r="E7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -647,8 +686,9 @@
         <v>4650.03</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>5229.44</v>
-      </c>
+        <v>4729.44</v>
+      </c>
+      <c r="E8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -665,6 +705,7 @@
       <c r="D9" s="3" t="n">
         <v>-79370.89999999999</v>
       </c>
+      <c r="E9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -681,6 +722,7 @@
       <c r="D10" s="3" t="n">
         <v>4042830.79</v>
       </c>
+      <c r="E10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -697,6 +739,7 @@
       <c r="D11" s="3" t="n">
         <v>1559808.16</v>
       </c>
+      <c r="E11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -713,6 +756,7 @@
       <c r="D12" s="3" t="n">
         <v>1888324.76</v>
       </c>
+      <c r="E12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -729,6 +773,7 @@
       <c r="D13" s="3" t="n">
         <v>124102.85</v>
       </c>
+      <c r="E13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -745,6 +790,7 @@
       <c r="D14" s="3" t="n">
         <v>5240690.11</v>
       </c>
+      <c r="E14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -761,6 +807,7 @@
       <c r="D15" s="3" t="n">
         <v>833591.47</v>
       </c>
+      <c r="E15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -777,6 +824,7 @@
       <c r="D16" s="3" t="n">
         <v>848224.47</v>
       </c>
+      <c r="E16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -793,11 +841,12 @@
       <c r="D17" s="3" t="n">
         <v>488129.72</v>
       </c>
+      <c r="E17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Lease liability - ST</t>
+          <t>Lease liability ST</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -807,13 +856,14 @@
         <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1240</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lease liability - LT</t>
+          <t>Lease liability LT</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -825,6 +875,7 @@
       <c r="D19" s="3" t="n">
         <v>1192003.83</v>
       </c>
+      <c r="E19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -841,6 +892,7 @@
       <c r="D20" s="3" t="n">
         <v>2630147.99</v>
       </c>
+      <c r="E20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -857,11 +909,12 @@
       <c r="D21" s="3" t="n">
         <v>1978718.87</v>
       </c>
+      <c r="E21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Retained earnings - prior</t>
+          <t>Retained earnings prior</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
@@ -871,8 +924,9 @@
         <v>6271867.35</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6231008.46</v>
-      </c>
+        <v>6232248.46</v>
+      </c>
+      <c r="E22" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -885,17 +939,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Income Statement</t>
         </is>
@@ -904,15 +959,20 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -924,15 +984,19 @@
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
+        <f>in_revenue_2026_01</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
         <f>in_revenue_2026_02</f>
         <v/>
       </c>
-      <c r="C3" s="3">
+      <c r="D3" s="4">
         <f>in_revenue_2026_03</f>
         <v/>
       </c>
-      <c r="D3" s="3">
+      <c r="E3" s="4">
         <f>in_revenue_2026_04</f>
         <v/>
       </c>
@@ -943,34 +1007,42 @@
           <t>COGS</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
+        <f>in_cogs_2026_01</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
         <f>in_cogs_2026_02</f>
         <v/>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="4">
         <f>in_cogs_2026_03</f>
         <v/>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="4">
         <f>in_cogs_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Gross profit</t>
         </is>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="7">
+        <f>in_revenue_2026_01+in_cogs_2026_01</f>
+        <v/>
+      </c>
+      <c r="C5" s="7">
         <f>in_revenue_2026_02+in_cogs_2026_02</f>
         <v/>
       </c>
-      <c r="C5" s="6">
+      <c r="D5" s="7">
         <f>in_revenue_2026_03+in_cogs_2026_03</f>
         <v/>
       </c>
-      <c r="D5" s="6">
+      <c r="E5" s="7">
         <f>in_revenue_2026_04+in_cogs_2026_04</f>
         <v/>
       </c>
@@ -981,15 +1053,19 @@
           <t>SG&amp;A</t>
         </is>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="4">
+        <f>in_sganda_2026_01</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
         <f>in_sganda_2026_02</f>
         <v/>
       </c>
-      <c r="C6" s="3">
+      <c r="D6" s="4">
         <f>in_sganda_2026_03</f>
         <v/>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="4">
         <f>in_sganda_2026_04</f>
         <v/>
       </c>
@@ -1000,15 +1076,19 @@
           <t>R&amp;D</t>
         </is>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="4">
+        <f>in_randd_2026_01</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
         <f>in_randd_2026_02</f>
         <v/>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="4">
         <f>in_randd_2026_03</f>
         <v/>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="4">
         <f>in_randd_2026_04</f>
         <v/>
       </c>
@@ -1019,34 +1099,42 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="4">
+        <f>in_depreciation_2026_01</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
         <f>in_depreciation_2026_02</f>
         <v/>
       </c>
-      <c r="C8" s="3">
+      <c r="D8" s="4">
         <f>in_depreciation_2026_03</f>
         <v/>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="4">
         <f>in_depreciation_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Operating income</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
+        <f>in_revenue_2026_01+in_cogs_2026_01+in_sganda_2026_01+in_randd_2026_01+in_depreciation_2026_01</f>
+        <v/>
+      </c>
+      <c r="C9" s="7">
         <f>in_revenue_2026_02+in_cogs_2026_02+in_sganda_2026_02+in_randd_2026_02+in_depreciation_2026_02</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="D9" s="7">
         <f>in_revenue_2026_03+in_cogs_2026_03+in_sganda_2026_03+in_randd_2026_03+in_depreciation_2026_03</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="E9" s="7">
         <f>in_revenue_2026_04+in_cogs_2026_04+in_sganda_2026_04+in_randd_2026_04+in_depreciation_2026_04</f>
         <v/>
       </c>
@@ -1057,15 +1145,19 @@
           <t>Interest income</t>
         </is>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="4">
+        <f>in_interest_income_2026_01</f>
+        <v/>
+      </c>
+      <c r="C10" s="4">
         <f>in_interest_income_2026_02</f>
         <v/>
       </c>
-      <c r="C10" s="3">
+      <c r="D10" s="4">
         <f>in_interest_income_2026_03</f>
         <v/>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="4">
         <f>in_interest_income_2026_04</f>
         <v/>
       </c>
@@ -1076,34 +1168,42 @@
           <t>Interest expense</t>
         </is>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="4">
+        <f>in_interest_expense_2026_01</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
         <f>in_interest_expense_2026_02</f>
         <v/>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="4">
         <f>in_interest_expense_2026_03</f>
         <v/>
       </c>
-      <c r="D11" s="3">
+      <c r="E11" s="4">
         <f>in_interest_expense_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Pretax income</t>
         </is>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="7">
+        <f>in_revenue_2026_01+in_cogs_2026_01+in_sganda_2026_01+in_randd_2026_01+in_depreciation_2026_01+in_interest_income_2026_01+in_interest_expense_2026_01</f>
+        <v/>
+      </c>
+      <c r="C12" s="7">
         <f>in_revenue_2026_02+in_cogs_2026_02+in_sganda_2026_02+in_randd_2026_02+in_depreciation_2026_02+in_interest_income_2026_02+in_interest_expense_2026_02</f>
         <v/>
       </c>
-      <c r="C12" s="6">
+      <c r="D12" s="7">
         <f>in_revenue_2026_03+in_cogs_2026_03+in_sganda_2026_03+in_randd_2026_03+in_depreciation_2026_03+in_interest_income_2026_03+in_interest_expense_2026_03</f>
         <v/>
       </c>
-      <c r="D12" s="6">
+      <c r="E12" s="7">
         <f>in_revenue_2026_04+in_cogs_2026_04+in_sganda_2026_04+in_randd_2026_04+in_depreciation_2026_04+in_interest_income_2026_04+in_interest_expense_2026_04</f>
         <v/>
       </c>
@@ -1114,34 +1214,42 @@
           <t>Tax expense</t>
         </is>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="4">
+        <f>in_tax_expense_2026_01</f>
+        <v/>
+      </c>
+      <c r="C13" s="4">
         <f>in_tax_expense_2026_02</f>
         <v/>
       </c>
-      <c r="C13" s="3">
+      <c r="D13" s="4">
         <f>in_tax_expense_2026_03</f>
         <v/>
       </c>
-      <c r="D13" s="3">
+      <c r="E13" s="4">
         <f>in_tax_expense_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Net income</t>
         </is>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="7">
+        <f>in_revenue_2026_01+in_cogs_2026_01+in_sganda_2026_01+in_randd_2026_01+in_depreciation_2026_01+in_interest_income_2026_01+in_interest_expense_2026_01+in_tax_expense_2026_01</f>
+        <v/>
+      </c>
+      <c r="C14" s="7">
         <f>in_revenue_2026_02+in_cogs_2026_02+in_sganda_2026_02+in_randd_2026_02+in_depreciation_2026_02+in_interest_income_2026_02+in_interest_expense_2026_02+in_tax_expense_2026_02</f>
         <v/>
       </c>
-      <c r="C14" s="6">
+      <c r="D14" s="7">
         <f>in_revenue_2026_03+in_cogs_2026_03+in_sganda_2026_03+in_randd_2026_03+in_depreciation_2026_03+in_interest_income_2026_03+in_interest_expense_2026_03+in_tax_expense_2026_03</f>
         <v/>
       </c>
-      <c r="D14" s="6">
+      <c r="E14" s="7">
         <f>in_revenue_2026_04+in_cogs_2026_04+in_sganda_2026_04+in_randd_2026_04+in_depreciation_2026_04+in_interest_income_2026_04+in_interest_expense_2026_04+in_tax_expense_2026_04</f>
         <v/>
       </c>
@@ -1157,17 +1265,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Balance Sheet</t>
         </is>
@@ -1176,15 +1285,20 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -1196,15 +1310,19 @@
           <t>Cash</t>
         </is>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
+        <f>in_cash_2026_01</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
         <f>in_cash_2026_02</f>
         <v/>
       </c>
-      <c r="C3" s="3">
+      <c r="D3" s="4">
         <f>in_cash_2026_03</f>
         <v/>
       </c>
-      <c r="D3" s="3">
+      <c r="E3" s="4">
         <f>in_cash_2026_04</f>
         <v/>
       </c>
@@ -1215,15 +1333,19 @@
           <t>AR</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
+        <f>in_ar_2026_01</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
         <f>in_ar_2026_02</f>
         <v/>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="4">
         <f>in_ar_2026_03</f>
         <v/>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="4">
         <f>in_ar_2026_04</f>
         <v/>
       </c>
@@ -1234,15 +1356,19 @@
           <t>Inventory</t>
         </is>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="4">
+        <f>in_inventory_2026_01</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
         <f>in_inventory_2026_02</f>
         <v/>
       </c>
-      <c r="C5" s="3">
+      <c r="D5" s="4">
         <f>in_inventory_2026_03</f>
         <v/>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="4">
         <f>in_inventory_2026_04</f>
         <v/>
       </c>
@@ -1253,15 +1379,19 @@
           <t>Prepaid expenses</t>
         </is>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="4">
+        <f>in_prepaid_expenses_2026_01</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
         <f>in_prepaid_expenses_2026_02</f>
         <v/>
       </c>
-      <c r="C6" s="3">
+      <c r="D6" s="4">
         <f>in_prepaid_expenses_2026_03</f>
         <v/>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="4">
         <f>in_prepaid_expenses_2026_04</f>
         <v/>
       </c>
@@ -1272,15 +1402,19 @@
           <t>PPE (net)</t>
         </is>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="4">
+        <f>in_ppe_2026_01</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
         <f>in_ppe_2026_02</f>
         <v/>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="4">
         <f>in_ppe_2026_03</f>
         <v/>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="4">
         <f>in_ppe_2026_04</f>
         <v/>
       </c>
@@ -1291,34 +1425,42 @@
           <t>Intangibles</t>
         </is>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="4">
+        <f>in_intangibles_2026_01</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
         <f>in_intangibles_2026_02</f>
         <v/>
       </c>
-      <c r="C8" s="3">
+      <c r="D8" s="4">
         <f>in_intangibles_2026_03</f>
         <v/>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="4">
         <f>in_intangibles_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Total assets</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
+        <f>in_cash_2026_01+in_ar_2026_01+in_inventory_2026_01+in_prepaid_expenses_2026_01+in_ppe_2026_01+in_intangibles_2026_01</f>
+        <v/>
+      </c>
+      <c r="C9" s="7">
         <f>in_cash_2026_02+in_ar_2026_02+in_inventory_2026_02+in_prepaid_expenses_2026_02+in_ppe_2026_02+in_intangibles_2026_02</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="D9" s="7">
         <f>in_cash_2026_03+in_ar_2026_03+in_inventory_2026_03+in_prepaid_expenses_2026_03+in_ppe_2026_03+in_intangibles_2026_03</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="E9" s="7">
         <f>in_cash_2026_04+in_ar_2026_04+in_inventory_2026_04+in_prepaid_expenses_2026_04+in_ppe_2026_04+in_intangibles_2026_04</f>
         <v/>
       </c>
@@ -1329,15 +1471,19 @@
           <t>AP</t>
         </is>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="4">
+        <f>in_ap_2026_01</f>
+        <v/>
+      </c>
+      <c r="C10" s="4">
         <f>in_ap_2026_02</f>
         <v/>
       </c>
-      <c r="C10" s="3">
+      <c r="D10" s="4">
         <f>in_ap_2026_03</f>
         <v/>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="4">
         <f>in_ap_2026_04</f>
         <v/>
       </c>
@@ -1348,15 +1494,19 @@
           <t>Accrued expenses</t>
         </is>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="4">
+        <f>in_accrued_expenses_2026_01</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
         <f>in_accrued_expenses_2026_02</f>
         <v/>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="4">
         <f>in_accrued_expenses_2026_03</f>
         <v/>
       </c>
-      <c r="D11" s="3">
+      <c r="E11" s="4">
         <f>in_accrued_expenses_2026_04</f>
         <v/>
       </c>
@@ -1364,18 +1514,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Lease liability - ST</t>
-        </is>
-      </c>
-      <c r="B12" s="3">
+          <t>Lease liability ST</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>in_lease_liability_st_2026_01</f>
+        <v/>
+      </c>
+      <c r="C12" s="4">
         <f>in_lease_liability_st_2026_02</f>
         <v/>
       </c>
-      <c r="C12" s="3">
+      <c r="D12" s="4">
         <f>in_lease_liability_st_2026_03</f>
         <v/>
       </c>
-      <c r="D12" s="3">
+      <c r="E12" s="4">
         <f>in_lease_liability_st_2026_04</f>
         <v/>
       </c>
@@ -1383,18 +1537,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Lease liability - LT</t>
-        </is>
-      </c>
-      <c r="B13" s="3">
+          <t>Lease liability LT</t>
+        </is>
+      </c>
+      <c r="B13" s="4">
+        <f>in_lease_liability_lt_2026_01</f>
+        <v/>
+      </c>
+      <c r="C13" s="4">
         <f>in_lease_liability_lt_2026_02</f>
         <v/>
       </c>
-      <c r="C13" s="3">
+      <c r="D13" s="4">
         <f>in_lease_liability_lt_2026_03</f>
         <v/>
       </c>
-      <c r="D13" s="3">
+      <c r="E13" s="4">
         <f>in_lease_liability_lt_2026_04</f>
         <v/>
       </c>
@@ -1405,34 +1563,42 @@
           <t>Debt</t>
         </is>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="4">
+        <f>in_debt_2026_01</f>
+        <v/>
+      </c>
+      <c r="C14" s="4">
         <f>in_debt_2026_02</f>
         <v/>
       </c>
-      <c r="C14" s="3">
+      <c r="D14" s="4">
         <f>in_debt_2026_03</f>
         <v/>
       </c>
-      <c r="D14" s="3">
+      <c r="E14" s="4">
         <f>in_debt_2026_04</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Total liabilities</t>
         </is>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="7">
+        <f>in_ap_2026_01+in_accrued_expenses_2026_01+in_lease_liability_st_2026_01+in_lease_liability_lt_2026_01+in_debt_2026_01</f>
+        <v/>
+      </c>
+      <c r="C15" s="7">
         <f>in_ap_2026_02+in_accrued_expenses_2026_02+in_lease_liability_st_2026_02+in_lease_liability_lt_2026_02+in_debt_2026_02</f>
         <v/>
       </c>
-      <c r="C15" s="6">
+      <c r="D15" s="7">
         <f>in_ap_2026_03+in_accrued_expenses_2026_03+in_lease_liability_st_2026_03+in_lease_liability_lt_2026_03+in_debt_2026_03</f>
         <v/>
       </c>
-      <c r="D15" s="6">
+      <c r="E15" s="7">
         <f>in_ap_2026_04+in_accrued_expenses_2026_04+in_lease_liability_st_2026_04+in_lease_liability_lt_2026_04+in_debt_2026_04</f>
         <v/>
       </c>
@@ -1443,15 +1609,19 @@
           <t>Common stock</t>
         </is>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="4">
+        <f>in_common_stock_2026_01</f>
+        <v/>
+      </c>
+      <c r="C16" s="4">
         <f>in_common_stock_2026_02</f>
         <v/>
       </c>
-      <c r="C16" s="3">
+      <c r="D16" s="4">
         <f>in_common_stock_2026_03</f>
         <v/>
       </c>
-      <c r="D16" s="3">
+      <c r="E16" s="4">
         <f>in_common_stock_2026_04</f>
         <v/>
       </c>
@@ -1462,54 +1632,66 @@
           <t>Retained earnings</t>
         </is>
       </c>
-      <c r="B17" s="3">
-        <f>in_retained_earnings_prior_2026_02+IS!B14</f>
-        <v/>
-      </c>
-      <c r="C17" s="3">
-        <f>in_retained_earnings_prior_2026_03+IS!C14</f>
-        <v/>
-      </c>
-      <c r="D17" s="3">
-        <f>in_retained_earnings_prior_2026_04+IS!D14</f>
+      <c r="B17" s="4">
+        <f>in_retained_earnings_prior_2026_01+IS!B14</f>
+        <v/>
+      </c>
+      <c r="C17" s="4">
+        <f>in_retained_earnings_prior_2026_02+IS!C14</f>
+        <v/>
+      </c>
+      <c r="D17" s="4">
+        <f>in_retained_earnings_prior_2026_03+IS!D14</f>
+        <v/>
+      </c>
+      <c r="E17" s="4">
+        <f>in_retained_earnings_prior_2026_04+IS!E14</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t>Total equity</t>
         </is>
       </c>
-      <c r="B18" s="6">
-        <f>in_common_stock_2026_02+in_retained_earnings_prior_2026_02+IS!B14</f>
-        <v/>
-      </c>
-      <c r="C18" s="6">
-        <f>in_common_stock_2026_03+in_retained_earnings_prior_2026_03+IS!C14</f>
-        <v/>
-      </c>
-      <c r="D18" s="6">
-        <f>in_common_stock_2026_04+in_retained_earnings_prior_2026_04+IS!D14</f>
+      <c r="B18" s="7">
+        <f>in_common_stock_2026_01+in_retained_earnings_prior_2026_01+IS!B14</f>
+        <v/>
+      </c>
+      <c r="C18" s="7">
+        <f>in_common_stock_2026_02+in_retained_earnings_prior_2026_02+IS!C14</f>
+        <v/>
+      </c>
+      <c r="D18" s="7">
+        <f>in_common_stock_2026_03+in_retained_earnings_prior_2026_03+IS!D14</f>
+        <v/>
+      </c>
+      <c r="E18" s="7">
+        <f>in_common_stock_2026_04+in_retained_earnings_prior_2026_04+IS!E14</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Check (A - L - E)</t>
         </is>
       </c>
-      <c r="B19" s="6">
+      <c r="B19" s="7">
         <f>B9-B15-B18</f>
         <v/>
       </c>
-      <c r="C19" s="6">
+      <c r="C19" s="7">
         <f>C9-C15-C18</f>
         <v/>
       </c>
-      <c r="D19" s="6">
+      <c r="D19" s="7">
         <f>D9-D15-D18</f>
+        <v/>
+      </c>
+      <c r="E19" s="7">
+        <f>E9-E15-E18</f>
         <v/>
       </c>
     </row>
@@ -1524,17 +1706,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Cash Flow</t>
         </is>
@@ -1543,15 +1726,20 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>2026-02</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>2026-04</t>
         </is>
@@ -1563,16 +1751,20 @@
           <t>Net income</t>
         </is>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="4">
         <f>IS!B14</f>
         <v/>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="4">
         <f>IS!C14</f>
         <v/>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="4">
         <f>IS!D14</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>IS!E14</f>
         <v/>
       </c>
     </row>
@@ -1582,15 +1774,19 @@
           <t>+ Depreciation</t>
         </is>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="4">
+        <f>-in_depreciation_2026_01</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
         <f>-in_depreciation_2026_02</f>
         <v/>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="4">
         <f>-in_depreciation_2026_03</f>
         <v/>
       </c>
-      <c r="D4" s="3">
+      <c r="E4" s="4">
         <f>-in_depreciation_2026_04</f>
         <v/>
       </c>
@@ -1601,11 +1797,15 @@
           <t>- Change in AR</t>
         </is>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="4">
+        <f>-(in_ar_2026_02-in_ar_2026_01)</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
         <f>-(in_ar_2026_03-in_ar_2026_02)</f>
         <v/>
       </c>
-      <c r="D5" s="3">
+      <c r="E5" s="4">
         <f>-(in_ar_2026_04-in_ar_2026_03)</f>
         <v/>
       </c>
@@ -1616,11 +1816,15 @@
           <t>- Change in Inventory</t>
         </is>
       </c>
-      <c r="C6" s="3">
+      <c r="C6" s="4">
+        <f>-(in_inventory_2026_02-in_inventory_2026_01)</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
         <f>-(in_inventory_2026_03-in_inventory_2026_02)</f>
         <v/>
       </c>
-      <c r="D6" s="3">
+      <c r="E6" s="4">
         <f>-(in_inventory_2026_04-in_inventory_2026_03)</f>
         <v/>
       </c>
@@ -1631,11 +1835,15 @@
           <t>+ Change in AP</t>
         </is>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="4">
+        <f>in_ap_2026_02-in_ap_2026_01</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
         <f>in_ap_2026_03-in_ap_2026_02</f>
         <v/>
       </c>
-      <c r="D7" s="3">
+      <c r="E7" s="4">
         <f>in_ap_2026_04-in_ap_2026_03</f>
         <v/>
       </c>
@@ -1646,31 +1854,39 @@
           <t>+ Change in Accrued</t>
         </is>
       </c>
-      <c r="C8" s="3">
+      <c r="C8" s="4">
+        <f>in_accrued_expenses_2026_02-in_accrued_expenses_2026_01</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
         <f>in_accrued_expenses_2026_03-in_accrued_expenses_2026_02</f>
         <v/>
       </c>
-      <c r="D8" s="3">
+      <c r="E8" s="4">
         <f>in_accrued_expenses_2026_04-in_accrued_expenses_2026_03</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Cash from operations</t>
         </is>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="7">
         <f>SUM(B3:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="7">
         <f>SUM(C3:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="7">
         <f>SUM(D3:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>SUM(E3:E8)</f>
         <v/>
       </c>
     </row>
@@ -1680,31 +1896,39 @@
           <t>- Change in PPE</t>
         </is>
       </c>
-      <c r="C10" s="3">
+      <c r="C10" s="4">
+        <f>-(in_ppe_2026_02-in_ppe_2026_01)</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
         <f>-(in_ppe_2026_03-in_ppe_2026_02)</f>
         <v/>
       </c>
-      <c r="D10" s="3">
+      <c r="E10" s="4">
         <f>-(in_ppe_2026_04-in_ppe_2026_03)</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Cash from investing</t>
         </is>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="7">
         <f>B10</f>
         <v/>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="7">
         <f>C10</f>
         <v/>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="7">
         <f>D10</f>
+        <v/>
+      </c>
+      <c r="E11" s="7">
+        <f>E10</f>
         <v/>
       </c>
     </row>
@@ -1714,11 +1938,15 @@
           <t>+ Change in Debt</t>
         </is>
       </c>
-      <c r="C12" s="3">
+      <c r="C12" s="4">
+        <f>in_debt_2026_02-in_debt_2026_01</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
         <f>in_debt_2026_03-in_debt_2026_02</f>
         <v/>
       </c>
-      <c r="D12" s="3">
+      <c r="E12" s="4">
         <f>in_debt_2026_04-in_debt_2026_03</f>
         <v/>
       </c>
@@ -1729,50 +1957,62 @@
           <t>+ Change in Lease liabilities</t>
         </is>
       </c>
-      <c r="C13" s="3">
+      <c r="C13" s="4">
+        <f>(in_lease_liability_st_2026_02-in_lease_liability_st_2026_01)+(in_lease_liability_lt_2026_02-in_lease_liability_lt_2026_01)</f>
+        <v/>
+      </c>
+      <c r="D13" s="4">
         <f>(in_lease_liability_st_2026_03-in_lease_liability_st_2026_02)+(in_lease_liability_lt_2026_03-in_lease_liability_lt_2026_02)</f>
         <v/>
       </c>
-      <c r="D13" s="3">
+      <c r="E13" s="4">
         <f>(in_lease_liability_st_2026_04-in_lease_liability_st_2026_03)+(in_lease_liability_lt_2026_04-in_lease_liability_lt_2026_03)</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Cash from financing</t>
         </is>
       </c>
-      <c r="B14" s="6">
+      <c r="B14" s="7">
         <f>SUM(B12:B13)</f>
         <v/>
       </c>
-      <c r="C14" s="6">
+      <c r="C14" s="7">
         <f>SUM(C12:C13)</f>
         <v/>
       </c>
-      <c r="D14" s="6">
+      <c r="D14" s="7">
         <f>SUM(D12:D13)</f>
         <v/>
       </c>
+      <c r="E14" s="7">
+        <f>SUM(E12:E13)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Net change in cash</t>
         </is>
       </c>
-      <c r="B15" s="6">
+      <c r="B15" s="7">
         <f>B8+B10+B14</f>
         <v/>
       </c>
-      <c r="C15" s="6">
+      <c r="C15" s="7">
         <f>C8+C10+C14</f>
         <v/>
       </c>
-      <c r="D15" s="6">
+      <c r="D15" s="7">
         <f>D8+D10+D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="7">
+        <f>E8+E10+E14</f>
         <v/>
       </c>
     </row>
@@ -1782,11 +2022,15 @@
           <t>Memo: Change in cash on BS</t>
         </is>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="4">
+        <f>in_cash_2026_02-in_cash_2026_01</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
         <f>in_cash_2026_03-in_cash_2026_02</f>
         <v/>
       </c>
-      <c r="D16" s="3">
+      <c r="E16" s="4">
         <f>in_cash_2026_04-in_cash_2026_03</f>
         <v/>
       </c>
@@ -1802,14 +2046,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Three-statement model - sample for vibecoding case</t>
         </is>
@@ -1821,21 +2065,21 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Inputs tab is where the automation script writes period numbers.</t>
+          <t>The Inputs tab holds period numbers. Jan/Feb/Mar are frozen actuals</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Each cell on Inputs has a defined name like in_revenue_2026_04 so</t>
+          <t>from prior monthly updates; April is empty and gets populated by</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>the script can write by name rather than by cell coordinate.</t>
+          <t>the automation script the analyst runs each month.</t>
         </is>
       </c>
     </row>
@@ -1845,14 +2089,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IS / BS / CF tabs reference Inputs through those names.</t>
+          <t>Each cell on Inputs has a defined name like in_revenue_2026_04 so</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Do not type numbers directly into IS, BS, or CF.</t>
+          <t>the script can write by name rather than by cell coordinate.</t>
         </is>
       </c>
     </row>
@@ -1862,33 +2106,74 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Sign convention on Inputs:</t>
+          <t>IS / BS / CF tabs reference Inputs through those names. Do not</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Revenue is positive, all expenses are negative.</t>
+          <t>type numbers directly into IS, BS, or CF.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Assets are positive, liabilities and equity are positive.</t>
-        </is>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Depreciation on Inputs is negative (an expense); the CF tab</t>
+          <t>Each new month, extend Inputs with one more column to the right</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>and add defined names for the new period before running the</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>script. The script does the rest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sign convention on Inputs:</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Revenue is positive, all expenses are negative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Assets are positive, liabilities and equity are positive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Depreciation on Inputs is negative (an expense); the CF tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t xml:space="preserve">  adds it back as a positive number.</t>
         </is>

</xml_diff>